<commit_message>
chore: update news radar report 2026-10-05
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-05.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-05.xlsx
@@ -477,27 +477,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Health Benefits Brokers Pursue New Cost-Containment Strategies Amid Rising Expenses</t>
+          <t>Rise in Cash-Pay GLP-1s Alters Employer Benefit Utilization Trends</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Insurance brokers and consultants are actively seeking alternative health plan strategies to combat soaring healthcare and pharmacy costs for employer clients. This shift highlights growing demand among self-funded employers for innovative PBM models, transparent pricing, and specialized cost-management solutions.</t>
+          <t>An increasing number of patients are bypassing traditional insurance and paying out-of-pocket for GLP-1 medications due to strict prior authorization and coverage exclusions by employers. This trend shifts utilization patterns outside employer-sponsored health plans, potentially impacting overall cost management strategies and employee satisfaction. Self-funded plan sponsors must evaluate whether cash-pay trends signal a need to redesign their obesity and diabetes benefit offerings.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Insurance Journal</t>
+          <t>Medical Economics</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 12:30:15 GMT</t>
+          <t>Mon, 05 Oct 2026 18:07:30 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPUUlhNmV4bFJXZmNXUjd5enJqSDJxSmtGbzZ0bm5JRkFsU09LdkhqdC1EYTV4eDlvSGw1RGJ2V29TUUF6cm52V0hpdm9kODJiZXpFMGhRT1hiSGdzMW5uX3lmeGc5VjFKaHhTZ3Q2RDhsS3JfN0FiTzBZcGFkMEZUcHUyTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbEVaZDBtWnh5ZTJqVnR5QVB3Nm9qTWFPaWFzalVRV3hfU0R4YkhSRjdVbHJMRXR2Z1d6TkVrcjE5Q29nVVNJNnJ3ODBVd0U5OUJLM05nNFZlWHdKZUpmcW5ZU2xvWUdsS09MZ2dROWRXaDhYZ2E4dU10cGFNdXhOWHE4LVVCYjhFa01VSlRpSk8?oc=5</t>
         </is>
       </c>
     </row>
@@ -507,27 +507,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FDA Approves Additional Manufacturing Capacity for Alvotech Humira Biosimilar</t>
+          <t>Bipartisan Congressional Scrutiny Intensifies Against Pharmacy Benefit Managers</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>The FDA has approved expanded manufacturing capacity for Alvotech's Humira biosimilar, bolstering supply chain stability for a key high-cost specialty drug. This increased manufacturing capacity supports broader market adoption of biosimilars, offering self-funded employer health plans enhanced opportunities to drive significant cost savings on specialty pharmacy spend.</t>
+          <t>Lawmakers from both major political parties are increasingly targeting pharmacy benefit managers (PBMs) for legislative reform, focusing on pricing practices and transparency. This bipartisan momentum signals potential federal policy changes that will impact how PBMs operate and report costs to self-funded employers. Self-funded health plan sponsors should monitor these developments as they may yield new transparency mandates and regulatory compliance requirements.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>marketscreener.com</t>
+          <t>KUOW</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 09:32:44 GMT</t>
+          <t>Mon, 05 Oct 2026 09:00:00 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPS2FIZjRWQjlxLVVZZDA1bS02MGNXTm91MUdWQ202SnJzX0N2X0UyQWJfbFNNUUJFMEFhQkFFY0o2MUVJa0lfamI5QVNZaERia3NrQkp2Yy1FdnJjMGpCTkZvTzIxMlRFRkxqelIyMDJxNkhnRHh0X2dZMU9ZMXlPejR5VEduUzQ5bWZqcVRaTFhHTFJnQXVVeDFVTkd4N3ZEcjE4ZXU2QVNtcXY2WFAyOHdEREZvZE1SMkNFUm9pMTRha0s0NTBIdFhYT3BQUTdkQTJZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQbE9qU1cyYm5pRGlMX0dzUFpuRzFyMl96ZHlTUEF6Z1pBcHl3RjQ5ejBNVWx6ek5NZVVaMU9Ub3JrOFMxbnZBQWlLdU0zbm55UURVa2hNbk1hMDJfaTEtcGRuOXhfbXlKbGhjNmJwSDhwbDZrMHNkbGw0UG12UUNWVHVFcU5NeHNiY0JIWXJrVjgyQzFuWVE2bnVPdHB0Z1g4ak5QS3Q1X3EwMHpndDRoUkNyUmdadw?oc=5</t>
         </is>
       </c>
     </row>
@@ -537,27 +537,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Bipartisan Congressional Scrutiny Mounts Against Pharmacy Benefit Managers</t>
+          <t>SHARx Warns Self-Funded Employers That Discounts Fail to Control Total Pharmacy Spending</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Lawmakers from both parties are increasingly uniting in their criticism and legislative efforts targeting pharmacy benefit managers (PBMs). This heightened bipartisan scrutiny signals a growing risk of federal reform regarding PBM pricing models, transparency, and rebate practices, directly impacting self-funded employer health plans.</t>
+          <t>Industry analysis highlights that relying solely on traditional pharmaceutical discounts is insufficient for self-funded employers managing escalating pharmacy costs. The report emphasizes the need for comprehensive cost-management strategies beyond standard rebate models to address the total cost of care. This directly impacts employer benefits planning and PBM evaluation criteria.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>NPR</t>
+          <t>PR Newswire</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 09:00:00 GMT</t>
+          <t>Mon, 05 Oct 2026 12:08:00 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQ2dzXzUxbXZEbmt2RVNpUEE3MldDejNUeGVuNVRZSlU0ZHhXUWVkc2NLOUhRTGV2YjQ2bmY3VUNrMTNRWlA1ZEg3WU96TC12SUdGVzQwRGpKY0lrbkE0bzBOeWo0Q1dYZ0Y0cUh3UmRkV1l2NnpaN1VRZTgtM3JWQktvbUJnYjJ2b3I3Q0RseHdoXzRCYmx6R3FHTFQ0cURxMnlrWGNOZkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQd210cVZjMElkYUlJVC1fVW5Za0MzYlBPSXg2UnNqR0xTdXRYUEFBeE43Z3ItSENTbXVjUXVlUldoTzVqZE53TzNxRzBSYW9GUkhNdlBYbkQ2dUtUT1EtYVFTWTNrUGRWMU51UlMyb25nX0ZNWjc1V2hhcDAzTlpWczN3dVM5U2swMWdRRGlSRFZCNTNDZGw2TXJtRFlJbi1XYXg3YUNCWFh0X01ONkk1RXJDYUZMVGFlU2JXMERhb1ZXbzFBeHpmc2F2SVoycExxTF9DVw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>